<commit_message>
Dashboard: Major overhaul to Premium Light Mode and fixed indicator data mapping
</commit_message>
<xml_diff>
--- a/Database Ekosistem Literat 2026.xlsx
+++ b/Database Ekosistem Literat 2026.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="160">
   <si>
     <t>lingkup</t>
   </si>
@@ -402,13 +402,19 @@
     <t>Kegiatan literasi meningkatkan keterampilan masyarakat sesuai kearifan lokal</t>
   </si>
   <si>
-    <t>timestamp</t>
-  </si>
-  <si>
-    <t>responden_nama</t>
-  </si>
-  <si>
-    <t>wilayah</t>
+    <t>Timestamp</t>
+  </si>
+  <si>
+    <t>User ID</t>
+  </si>
+  <si>
+    <t>Lingkup</t>
+  </si>
+  <si>
+    <t>Nama</t>
+  </si>
+  <si>
+    <t>Wilayah</t>
   </si>
   <si>
     <t>S1</t>
@@ -456,55 +462,34 @@
     <t>M5</t>
   </si>
   <si>
+    <t>2026-04-23T17:22:22.052Z</t>
+  </si>
+  <si>
+    <t>USR-1776964942052-FJCBK7XIN</t>
+  </si>
+  <si>
+    <t>BUDA</t>
+  </si>
+  <si>
+    <t>BOGOR</t>
+  </si>
+  <si>
+    <t>Skor (0-100)</t>
+  </si>
+  <si>
+    <t>Index (0.00-4.00)</t>
+  </si>
+  <si>
+    <t>Kategori</t>
+  </si>
+  <si>
+    <t>Perlu Perhatian</t>
+  </si>
+  <si>
+    <t>total_responden</t>
+  </si>
+  <si>
     <t>avg_score</t>
-  </si>
-  <si>
-    <t>S1_val</t>
-  </si>
-  <si>
-    <t>S2_val</t>
-  </si>
-  <si>
-    <t>S3_val</t>
-  </si>
-  <si>
-    <t>S4_val</t>
-  </si>
-  <si>
-    <t>S5_val</t>
-  </si>
-  <si>
-    <t>K1_val</t>
-  </si>
-  <si>
-    <t>K2_val</t>
-  </si>
-  <si>
-    <t>K3_val</t>
-  </si>
-  <si>
-    <t>K4_val</t>
-  </si>
-  <si>
-    <t>K5_val</t>
-  </si>
-  <si>
-    <t>M1_val</t>
-  </si>
-  <si>
-    <t>M2_val</t>
-  </si>
-  <si>
-    <t>M3_val</t>
-  </si>
-  <si>
-    <t>M4_val</t>
-  </si>
-  <si>
-    <t>M5_val</t>
-  </si>
-  <si>
-    <t>total_responden</t>
   </si>
   <si>
     <t>target_responden</t>
@@ -1755,58 +1740,78 @@
         <v>127</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K1" s="4" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="L1" s="4" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M1" s="4" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="N1" s="4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O1" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="P1" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="Q1" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="R1" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="S1" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
+      </c>
+      <c r="T1" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1820,64 +1825,53 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="6.63"/>
+    <col customWidth="1" min="2" max="2" width="6.88"/>
+    <col customWidth="1" min="3" max="3" width="10.25"/>
+    <col customWidth="1" min="4" max="4" width="13.75"/>
+    <col customWidth="1" min="5" max="5" width="7.25"/>
+    <col customWidth="1" min="6" max="6" width="9.13"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>127</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="F1" s="4" t="s">
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="D2" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>147</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>148</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="L1" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="N1" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>156</v>
-      </c>
-      <c r="P1" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q1" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="R1" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="S1" s="4" t="s">
-        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -1897,13 +1891,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2">
@@ -1935,10 +1929,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="4" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix: Corrected indicator mapping for all 45 fields and fixed dashboard score calculation
</commit_message>
<xml_diff>
--- a/Database Ekosistem Literat 2026.xlsx
+++ b/Database Ekosistem Literat 2026.xlsx
@@ -417,70 +417,70 @@
     <t>Wilayah</t>
   </si>
   <si>
-    <t>S1</t>
-  </si>
-  <si>
-    <t>S2</t>
-  </si>
-  <si>
-    <t>S3</t>
-  </si>
-  <si>
-    <t>S4</t>
-  </si>
-  <si>
-    <t>S5</t>
-  </si>
-  <si>
-    <t>K1</t>
-  </si>
-  <si>
-    <t>K2</t>
-  </si>
-  <si>
-    <t>K3</t>
-  </si>
-  <si>
-    <t>K4</t>
-  </si>
-  <si>
-    <t>K5</t>
-  </si>
-  <si>
-    <t>M1</t>
-  </si>
-  <si>
-    <t>M2</t>
-  </si>
-  <si>
-    <t>M3</t>
-  </si>
-  <si>
-    <t>M4</t>
-  </si>
-  <si>
-    <t>M5</t>
-  </si>
-  <si>
-    <t>2026-04-23T17:22:22.052Z</t>
-  </si>
-  <si>
-    <t>USR-1776964942052-FJCBK7XIN</t>
-  </si>
-  <si>
-    <t>BUDA</t>
+    <t>S1.1</t>
+  </si>
+  <si>
+    <t>S1.2</t>
+  </si>
+  <si>
+    <t>S1.3</t>
+  </si>
+  <si>
+    <t>S1.4</t>
+  </si>
+  <si>
+    <t>S1.5</t>
+  </si>
+  <si>
+    <t>K1.1</t>
+  </si>
+  <si>
+    <t>K1.2</t>
+  </si>
+  <si>
+    <t>K1.3</t>
+  </si>
+  <si>
+    <t>K1.4</t>
+  </si>
+  <si>
+    <t>K1.5</t>
+  </si>
+  <si>
+    <t>M1.1</t>
+  </si>
+  <si>
+    <t>M1.2</t>
+  </si>
+  <si>
+    <t>M1.3</t>
+  </si>
+  <si>
+    <t>M1.4</t>
+  </si>
+  <si>
+    <t>M1.5</t>
+  </si>
+  <si>
+    <t>2026-04-23T17:36:56.635Z</t>
+  </si>
+  <si>
+    <t>USR-1776965816635-MRNRKZO5P</t>
+  </si>
+  <si>
+    <t>BUDI</t>
   </si>
   <si>
     <t>BOGOR</t>
   </si>
   <si>
-    <t>Skor (0-100)</t>
-  </si>
-  <si>
-    <t>Index (0.00-4.00)</t>
-  </si>
-  <si>
-    <t>Kategori</t>
+    <t>Total Score (%)</t>
+  </si>
+  <si>
+    <t>Index (4.00)</t>
+  </si>
+  <si>
+    <t>Category</t>
   </si>
   <si>
     <t>Perlu Perhatian</t>
@@ -505,7 +505,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -517,17 +517,29 @@
       <name val="Arial"/>
     </font>
     <font>
+      <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="lightGray"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF3F4F6"/>
+        <bgColor rgb="FFF3F4F6"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -536,7 +548,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -545,7 +557,13 @@
       <alignment shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="9" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -1798,20 +1816,29 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="C2" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="C2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="5" t="s">
         <v>150</v>
+      </c>
+      <c r="F2" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="G2" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="H2" s="6">
+        <v>3.0</v>
       </c>
     </row>
   </sheetData>
@@ -1855,22 +1882,22 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C2" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="D2" s="4">
-        <v>0.0</v>
-      </c>
-      <c r="E2" s="4" t="s">
+      <c r="B2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="5">
+        <v>66.7</v>
+      </c>
+      <c r="D2" s="5">
+        <v>0.67</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="5" t="s">
         <v>147</v>
       </c>
     </row>
@@ -1887,31 +1914,31 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>156</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>157</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1928,10 +1955,10 @@
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>159</v>
       </c>
     </row>

</xml_diff>